<commit_message>
feat: add NRR (net revenue retention) to unit economics
</commit_message>
<xml_diff>
--- a/outputs/unit_economics_table.xlsx
+++ b/outputs/unit_economics_table.xlsx
@@ -523,7 +523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -534,6 +534,7 @@
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -591,6 +592,11 @@
           <t>LTV:MRR Ratio</t>
         </is>
       </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>NRR T12M (%)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -621,6 +627,11 @@
       <c r="H5" s="5" t="n">
         <v>3.2</v>
       </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>248.3%</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -651,6 +662,11 @@
       <c r="H6" s="7" t="n">
         <v>2.5</v>
       </c>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>298.5%</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
@@ -681,11 +697,16 @@
       <c r="H7" s="9" t="n">
         <v>2.7</v>
       </c>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>329.5%</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>